<commit_message>
removed news feature + cleaned stock mode
</commit_message>
<xml_diff>
--- a/stock_comparison.xlsx
+++ b/stock_comparison.xlsx
@@ -11,8 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financials" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyst Ratings" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -495,9 +494,9 @@
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,17 +512,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>AAPL</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>MRVL</t>
         </is>
       </c>
     </row>
@@ -537,13 +536,13 @@
         <v>202.06</v>
       </c>
       <c r="C2" t="n">
-        <v>273.05</v>
+        <v>147.84</v>
       </c>
       <c r="D2" t="n">
         <v>316.99</v>
       </c>
       <c r="E2" t="n">
-        <v>147.84</v>
+        <v>273.05</v>
       </c>
     </row>
     <row r="3">
@@ -556,13 +555,13 @@
         <v>4911068086272</v>
       </c>
       <c r="C3" t="n">
-        <v>4013268402176</v>
+        <v>129279901696</v>
       </c>
       <c r="D3" t="n">
         <v>854932258816</v>
       </c>
       <c r="E3" t="n">
-        <v>129279901696</v>
+        <v>4013268402176</v>
       </c>
     </row>
     <row r="4">
@@ -575,13 +574,13 @@
         <v>212.19</v>
       </c>
       <c r="C4" t="n">
-        <v>288.62</v>
+        <v>149.58</v>
       </c>
       <c r="D4" t="n">
         <v>337.25</v>
       </c>
       <c r="E4" t="n">
-        <v>149.58</v>
+        <v>288.62</v>
       </c>
     </row>
     <row r="5">
@@ -594,13 +593,13 @@
         <v>97.28</v>
       </c>
       <c r="C5" t="n">
-        <v>193.25</v>
+        <v>49.78</v>
       </c>
       <c r="D5" t="n">
         <v>231.37</v>
       </c>
       <c r="E5" t="n">
-        <v>49.78</v>
+        <v>193.25</v>
       </c>
     </row>
     <row r="6">
@@ -613,13 +612,13 @@
         <v>118513377</v>
       </c>
       <c r="C6" t="n">
-        <v>34667241</v>
+        <v>38692791</v>
       </c>
       <c r="D6" t="n">
         <v>6280698</v>
       </c>
       <c r="E6" t="n">
-        <v>38692791</v>
+        <v>34667241</v>
       </c>
     </row>
     <row r="7">
@@ -632,13 +631,13 @@
         <v>175294618</v>
       </c>
       <c r="C7" t="n">
-        <v>46163596</v>
+        <v>20781681</v>
       </c>
       <c r="D7" t="n">
         <v>10510318</v>
       </c>
       <c r="E7" t="n">
-        <v>20781681</v>
+        <v>46163596</v>
       </c>
     </row>
     <row r="8">
@@ -651,13 +650,13 @@
         <v>2.335</v>
       </c>
       <c r="C8" t="n">
-        <v>1.109</v>
+        <v>1.822</v>
       </c>
       <c r="D8" t="n">
         <v>1.043</v>
       </c>
       <c r="E8" t="n">
-        <v>1.822</v>
+        <v>1.109</v>
       </c>
     </row>
     <row r="9">
@@ -670,13 +669,13 @@
         <v>0.02</v>
       </c>
       <c r="C9" t="n">
-        <v>0.38</v>
+        <v>0.16</v>
       </c>
       <c r="D9" t="n">
         <v>1.89</v>
       </c>
       <c r="E9" t="n">
-        <v>0.16</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="10">
@@ -689,13 +688,13 @@
         <v>1773187200</v>
       </c>
       <c r="C10" t="n">
-        <v>1770595200</v>
+        <v>1775779200</v>
       </c>
       <c r="D10" t="n">
         <v>1775433600</v>
       </c>
       <c r="E10" t="n">
-        <v>1775779200</v>
+        <v>1770595200</v>
       </c>
     </row>
     <row r="11">
@@ -708,13 +707,13 @@
         <v>24300000000</v>
       </c>
       <c r="C11" t="n">
-        <v>14681140000</v>
+        <v>874458245</v>
       </c>
       <c r="D11" t="n">
         <v>2679500000</v>
       </c>
       <c r="E11" t="n">
-        <v>874458245</v>
+        <v>14681140000</v>
       </c>
     </row>
     <row r="12">
@@ -754,13 +753,13 @@
         <v>0.0121</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0086</v>
+        <v>0.0381</v>
       </c>
       <c r="D13" t="n">
         <v>0.0098</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0381</v>
+        <v>0.0086</v>
       </c>
     </row>
   </sheetData>
@@ -779,9 +778,9 @@
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -797,17 +796,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>AAPL</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>MRVL</t>
         </is>
       </c>
     </row>
@@ -821,13 +820,13 @@
         <v>41.152752</v>
       </c>
       <c r="C2" t="n">
-        <v>34.607098</v>
+        <v>48</v>
       </c>
       <c r="D2" t="n">
         <v>15.174246</v>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>34.607098</v>
       </c>
     </row>
     <row r="3">
@@ -840,13 +839,13 @@
         <v>17.97818</v>
       </c>
       <c r="C3" t="n">
-        <v>29.136738</v>
+        <v>27.253773</v>
       </c>
       <c r="D3" t="n">
         <v>13.482837</v>
       </c>
       <c r="E3" t="n">
-        <v>27.253773</v>
+        <v>29.136738</v>
       </c>
     </row>
     <row r="4">
@@ -859,13 +858,13 @@
         <v>0.72</v>
       </c>
       <c r="C4" t="n">
-        <v>2.43</v>
+        <v>1.64</v>
       </c>
       <c r="D4" t="n">
         <v>1.67</v>
       </c>
       <c r="E4" t="n">
-        <v>1.64</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="5">
@@ -878,13 +877,13 @@
         <v>22.742954</v>
       </c>
       <c r="C5" t="n">
-        <v>9.212837</v>
+        <v>15.776231</v>
       </c>
       <c r="D5" t="n">
         <v>4.925888</v>
       </c>
       <c r="E5" t="n">
-        <v>15.776231</v>
+        <v>9.212837</v>
       </c>
     </row>
     <row r="6">
@@ -897,13 +896,13 @@
         <v>31.220642</v>
       </c>
       <c r="C6" t="n">
-        <v>45.523506</v>
+        <v>8.754663000000001</v>
       </c>
       <c r="D6" t="n">
         <v>2.469154</v>
       </c>
       <c r="E6" t="n">
-        <v>8.754663000000001</v>
+        <v>45.523506</v>
       </c>
     </row>
     <row r="7">
@@ -916,15 +915,15 @@
         <v>36.47</v>
       </c>
       <c r="C7" t="n">
+        <v>49.975</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
         <v>26.372</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>49.975</v>
       </c>
     </row>
     <row r="8">
@@ -937,13 +936,13 @@
         <v>22.501</v>
       </c>
       <c r="C8" t="n">
-        <v>9.256</v>
+        <v>16.036</v>
       </c>
       <c r="D8" t="n">
         <v>1.827</v>
       </c>
       <c r="E8" t="n">
-        <v>16.036</v>
+        <v>9.256</v>
       </c>
     </row>
     <row r="9">
@@ -956,13 +955,13 @@
         <v>4858914013184</v>
       </c>
       <c r="C9" t="n">
-        <v>4032287211520</v>
+        <v>131408011264</v>
       </c>
       <c r="D9" t="n">
         <v>317048717312</v>
       </c>
       <c r="E9" t="n">
-        <v>131408011264</v>
+        <v>4032287211520</v>
       </c>
     </row>
   </sheetData>
@@ -981,9 +980,9 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -999,17 +998,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>AAPL</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>MRVL</t>
         </is>
       </c>
     </row>
@@ -1023,13 +1022,13 @@
         <v>215938007040</v>
       </c>
       <c r="C2" t="n">
-        <v>435617005568</v>
+        <v>8194599936</v>
       </c>
       <c r="D2" t="n">
         <v>173559005184</v>
       </c>
       <c r="E2" t="n">
-        <v>8194599936</v>
+        <v>435617005568</v>
       </c>
     </row>
     <row r="3">
@@ -1042,13 +1041,13 @@
         <v>0.732</v>
       </c>
       <c r="C3" t="n">
-        <v>0.157</v>
+        <v>0.221</v>
       </c>
       <c r="D3" t="n">
         <v>0.127</v>
       </c>
       <c r="E3" t="n">
-        <v>0.221</v>
+        <v>0.157</v>
       </c>
     </row>
     <row r="4">
@@ -1061,13 +1060,13 @@
         <v>0.71068</v>
       </c>
       <c r="C4" t="n">
-        <v>0.47325</v>
+        <v>0.51023996</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.51023996</v>
+        <v>0.47325</v>
       </c>
     </row>
     <row r="5">
@@ -1080,13 +1079,13 @@
         <v>0.55603004</v>
       </c>
       <c r="C5" t="n">
-        <v>0.27037</v>
+        <v>0.32584</v>
       </c>
       <c r="D5" t="n">
         <v>0.33936</v>
       </c>
       <c r="E5" t="n">
-        <v>0.32584</v>
+        <v>0.27037</v>
       </c>
     </row>
     <row r="6">
@@ -1099,13 +1098,13 @@
         <v>4.91</v>
       </c>
       <c r="C6" t="n">
-        <v>7.89</v>
+        <v>3.08</v>
       </c>
       <c r="D6" t="n">
         <v>20.89</v>
       </c>
       <c r="E6" t="n">
-        <v>3.08</v>
+        <v>7.89</v>
       </c>
     </row>
     <row r="7">
@@ -1118,13 +1117,13 @@
         <v>0.956</v>
       </c>
       <c r="C7" t="n">
-        <v>0.183</v>
+        <v>1.063</v>
       </c>
       <c r="D7" t="n">
         <v>0.172</v>
       </c>
       <c r="E7" t="n">
-        <v>1.063</v>
+        <v>0.183</v>
       </c>
     </row>
     <row r="8">
@@ -1137,15 +1136,15 @@
         <v>7.255</v>
       </c>
       <c r="C8" t="n">
+        <v>33.479</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
         <v>102.63</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>33.479</v>
       </c>
     </row>
     <row r="9">
@@ -1158,15 +1157,15 @@
         <v>58128998400</v>
       </c>
       <c r="C9" t="n">
+        <v>1442787456</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
         <v>106312753152</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>1442787456</v>
       </c>
     </row>
     <row r="10">
@@ -1179,13 +1178,13 @@
         <v>1.01485</v>
       </c>
       <c r="C10" t="n">
-        <v>1.5202099</v>
+        <v>0.19253999</v>
       </c>
       <c r="D10" t="n">
         <v>0.16465001</v>
       </c>
       <c r="E10" t="n">
-        <v>0.19253999</v>
+        <v>1.5202099</v>
       </c>
     </row>
     <row r="11">
@@ -1198,13 +1197,13 @@
         <v>0.51188</v>
       </c>
       <c r="C11" t="n">
-        <v>0.24377</v>
+        <v>0.039389998</v>
       </c>
       <c r="D11" t="n">
         <v>0.01272</v>
       </c>
       <c r="E11" t="n">
-        <v>0.039389998</v>
+        <v>0.24377</v>
       </c>
     </row>
   </sheetData>
@@ -1295,26 +1294,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" t="n">
         <v>7</v>
-      </c>
-      <c r="C3" t="n">
-        <v>24</v>
-      </c>
-      <c r="D3" t="n">
-        <v>14</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -1345,26 +1344,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1379,620 +1378,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>MRVL</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>1970-01-01</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Could not fetch article</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData/>

</xml_diff>

<commit_message>
fixed technicals and earnings
</commit_message>
<xml_diff>
--- a/stock_comparison.xlsx
+++ b/stock_comparison.xlsx
@@ -162,7 +162,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>8</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9525000" cy="5715000"/>
@@ -505,15 +505,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -547,6 +548,11 @@
           <t>PATH</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>RBRK</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -555,19 +561,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>200.2001</v>
+        <v>199.34</v>
       </c>
       <c r="C2" t="n">
-        <v>265.78</v>
+        <v>266.35</v>
       </c>
       <c r="D2" t="n">
-        <v>315.285</v>
+        <v>314.36</v>
       </c>
       <c r="E2" t="n">
-        <v>151.97</v>
+        <v>151.21</v>
       </c>
       <c r="F2" t="n">
-        <v>10.9099</v>
+        <v>10.7501</v>
+      </c>
+      <c r="G2" t="n">
+        <v>54.43</v>
       </c>
     </row>
     <row r="3">
@@ -577,19 +586,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4865863450624</v>
+        <v>4844958515200</v>
       </c>
       <c r="C3" t="n">
-        <v>3906414575616</v>
+        <v>3914792697856</v>
       </c>
       <c r="D3" t="n">
-        <v>850333859840</v>
+        <v>847839100928</v>
       </c>
       <c r="E3" t="n">
-        <v>132891418624</v>
+        <v>132226834432</v>
       </c>
       <c r="F3" t="n">
-        <v>5834065408</v>
+        <v>5748612608</v>
+      </c>
+      <c r="G3" t="n">
+        <v>11202229248</v>
       </c>
     </row>
     <row r="4">
@@ -613,6 +625,9 @@
       <c r="F4" t="n">
         <v>19.84</v>
       </c>
+      <c r="G4" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -635,6 +650,9 @@
       <c r="F5" t="n">
         <v>9.279999999999999</v>
       </c>
+      <c r="G5" t="n">
+        <v>42.25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -643,19 +661,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54887974</v>
+        <v>66822176</v>
       </c>
       <c r="C6" t="n">
-        <v>21873997</v>
+        <v>27805225</v>
       </c>
       <c r="D6" t="n">
-        <v>2624589</v>
+        <v>3091261</v>
       </c>
       <c r="E6" t="n">
-        <v>21662863</v>
+        <v>24320793</v>
       </c>
       <c r="F6" t="n">
-        <v>13552250</v>
+        <v>17926073</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2325391</v>
       </c>
     </row>
     <row r="7">
@@ -679,6 +700,9 @@
       <c r="F7" t="n">
         <v>32000650</v>
       </c>
+      <c r="G7" t="n">
+        <v>4255631</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -701,6 +725,11 @@
       <c r="F8" t="n">
         <v>1.025</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -725,6 +754,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -749,6 +783,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -771,6 +810,9 @@
       <c r="F11" t="n">
         <v>459231166</v>
       </c>
+      <c r="G11" t="n">
+        <v>160938033</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -803,6 +845,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -824,6 +871,71 @@
       </c>
       <c r="F13" t="n">
         <v>0.2555</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.08890000000000001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Analyst Price Target</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>268.6148</v>
+      </c>
+      <c r="C14" t="n">
+        <v>297.4555</v>
+      </c>
+      <c r="D14" t="n">
+        <v>338.45456</v>
+      </c>
+      <c r="E14" t="n">
+        <v>126.95039</v>
+      </c>
+      <c r="F14" t="n">
+        <v>13.805</v>
+      </c>
+      <c r="G14" t="n">
+        <v>85.79167</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Upside/Downside</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>+34.8%</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>+11.7%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>+7.7%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>-16.0%</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>+28.4%</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>+57.6%</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -837,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -846,6 +958,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -879,6 +992,11 @@
           <t>PATH</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>RBRK</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -887,19 +1005,24 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40.773952</v>
+        <v>40.598778</v>
       </c>
       <c r="C2" t="n">
-        <v>33.68568</v>
+        <v>33.757923</v>
       </c>
       <c r="D2" t="n">
-        <v>15.0926285</v>
+        <v>15.048348</v>
       </c>
       <c r="E2" t="n">
-        <v>49.34091</v>
+        <v>49.09416</v>
       </c>
       <c r="F2" t="n">
-        <v>20.980577</v>
+        <v>20.673271</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -909,19 +1032,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17.812696</v>
+        <v>17.73617</v>
       </c>
       <c r="C3" t="n">
-        <v>28.360968</v>
+        <v>28.421793</v>
       </c>
       <c r="D3" t="n">
-        <v>13.410317</v>
+        <v>13.370973</v>
       </c>
       <c r="E3" t="n">
-        <v>28.015123</v>
+        <v>27.875021</v>
       </c>
       <c r="F3" t="n">
-        <v>12.171337</v>
+        <v>11.993061</v>
+      </c>
+      <c r="G3" t="n">
+        <v>93.30911</v>
       </c>
     </row>
     <row r="4">
@@ -945,6 +1071,11 @@
       <c r="F4" t="n">
         <v>0.36</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -953,19 +1084,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22.533613</v>
+        <v>22.436804</v>
       </c>
       <c r="C5" t="n">
-        <v>8.967544</v>
+        <v>8.986776000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>4.8993936</v>
+        <v>4.8850193</v>
       </c>
       <c r="E5" t="n">
-        <v>16.21695</v>
+        <v>16.135849</v>
       </c>
       <c r="F5" t="n">
-        <v>3.6223562</v>
+        <v>3.5692987</v>
+      </c>
+      <c r="G5" t="n">
+        <v>8.511096999999999</v>
       </c>
     </row>
     <row r="6">
@@ -975,19 +1109,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30.933266</v>
+        <v>30.80037</v>
       </c>
       <c r="C6" t="n">
-        <v>44.311436</v>
+        <v>44.406467</v>
       </c>
       <c r="D6" t="n">
-        <v>2.455873</v>
+        <v>2.4486678</v>
       </c>
       <c r="E6" t="n">
-        <v>8.999230000000001</v>
+        <v>8.954226</v>
       </c>
       <c r="F6" t="n">
-        <v>2.8132799</v>
+        <v>2.7720733</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-21.187233</v>
       </c>
     </row>
     <row r="7">
@@ -1013,6 +1150,9 @@
       <c r="F7" t="n">
         <v>54.827</v>
       </c>
+      <c r="G7" t="n">
+        <v>-32.273</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1035,6 +1175,9 @@
       <c r="F8" t="n">
         <v>2.571</v>
       </c>
+      <c r="G8" t="n">
+        <v>7.851</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1056,6 +1199,9 @@
       </c>
       <c r="F9" t="n">
         <v>4141374976</v>
+      </c>
+      <c r="G9" t="n">
+        <v>10333908992</v>
       </c>
     </row>
   </sheetData>
@@ -1069,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1078,6 +1224,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1111,6 +1258,11 @@
           <t>PATH</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>RBRK</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1133,6 +1285,9 @@
       <c r="F2" t="n">
         <v>1610572032</v>
       </c>
+      <c r="G2" t="n">
+        <v>1316190976</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1155,6 +1310,9 @@
       <c r="F3" t="n">
         <v>0.136</v>
       </c>
+      <c r="G3" t="n">
+        <v>0.463</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1177,6 +1335,9 @@
       <c r="F4" t="n">
         <v>0.83242</v>
       </c>
+      <c r="G4" t="n">
+        <v>0.80103</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1199,6 +1360,9 @@
       <c r="F5" t="n">
         <v>0.1753</v>
       </c>
+      <c r="G5" t="n">
+        <v>-0.26503</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1221,6 +1385,9 @@
       <c r="F6" t="n">
         <v>0.52</v>
       </c>
+      <c r="G6" t="n">
+        <v>-1.78</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1243,6 +1410,11 @@
       <c r="F7" t="n">
         <v>1.057</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1267,6 +1439,11 @@
       <c r="F8" t="n">
         <v>3.901</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1291,6 +1468,9 @@
       <c r="F9" t="n">
         <v>473554368</v>
       </c>
+      <c r="G9" t="n">
+        <v>392845120</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1313,6 +1493,11 @@
       <c r="F10" t="n">
         <v>0.14374</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1334,6 +1519,9 @@
       </c>
       <c r="F11" t="n">
         <v>0.01265</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.10306</v>
       </c>
     </row>
   </sheetData>
@@ -1347,7 +1535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1521,6 +1709,31 @@
         <v>18</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RBRK</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>23</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1533,13 +1746,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1600,79 +1813,268 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>89.8</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>RSI of 89.8 - overbought territory</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Earnings Trend</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>3 declining qtrs</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>EPS had declined 3 consecutive quarters - watch for deteriorating fundamentals</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>PEG Ratio</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>2.43</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>PEG of 2.43 suggests growth may be fully priced in</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Caution</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Earnings Trend</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>2 declining qtrs</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>EPS had declined 2 consecutive quarters - watch for deteriorating fundamentals</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>74.1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>RSI of 74.1 - overbought territory</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Caution</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>MRVL</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>52W High</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>$151.97</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Trading within 2% of 52-week high ($154.95) - at extreme high</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>97.5</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>RSI of 97.5 - overbought territory</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Caution</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Earnings Trend</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>2 declining qtrs</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>EPS had declined 2 consecutive quarters - watch for deteriorating fundamentals</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>PATH</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Short % of Float</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>25.6%</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>25.6% of loat is shorted - heavily shorted, elevated risk</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>PATH</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Earnings Trend</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>2 declining qtrs</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>EPS had declined 2 consecutive quarters - watch for deteriorating fundamentals</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>RBRK</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Earnings Trend</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>2 declining qtrs</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>EPS had declined 2 consecutive quarters - watch for deteriorating fundamentals</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Warning</t>
         </is>

</xml_diff>